<commit_message>
Test plan builder: read an FRS priority stated as High / Medium / Low; rebuild the Claims plan
The Claims FRS writes its priorities as "High (BRD p.21)", which the builder
mapped to Medium on the Test Conditions sheet. The builder now accepts the level
stated directly; the Claims conditions show High and the finding that recorded
the mismatch is withdrawn.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01W3DAuLtsQmip7EuxjJCCtN
</commit_message>
<xml_diff>
--- a/docs/deliverables/out/TestPlans/BIBS_TestPlan_BRD-07_Claims_v1.0.xlsx
+++ b/docs/deliverables/out/TestPlans/BIBS_TestPlan_BRD-07_Claims_v1.0.xlsx
@@ -36,7 +36,7 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="7">'Test Data'!$4:$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Roles and Access'!$A$4:$M$89</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="8">'Roles and Access'!$4:$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'FRS Findings'!$A$4:$D$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'FRS Findings'!$A$4:$D$11</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="9">'FRS Findings'!$4:$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1022,7 +1022,7 @@
         </is>
       </c>
       <c r="D28" s="12" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="30">
@@ -1134,7 +1134,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1325,48 +1325,26 @@
       </c>
       <c r="B11" s="12" t="inlineStr">
         <is>
-          <t>FR-CL-002</t>
+          <t>FR-CL-016</t>
         </is>
       </c>
       <c r="C11" s="12" t="inlineStr">
         <is>
-          <t>The FR is "High (BRD p.21)", a value the test plan builder does not map to High; the Test Conditions sheet shows the Claims conditions of every "High (BRD p.21)" FR as Medium while the cases carry High. The same applies to the other FRs with this priority.</t>
+          <t>The meaning of the claims authorization code and any TL / TH override are open (CLQ01); the FRS tests only that the button is disabled while premium is unpaid.</t>
         </is>
       </c>
       <c r="D11" s="12" t="inlineStr">
         <is>
-          <t>Write the BRD priority as "High" or "Must have" in the fr blocks (keeping the page note in the trace), or extend the builder mapping.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="12" t="inlineStr">
-        <is>
-          <t>TF-CL-08</t>
-        </is>
-      </c>
-      <c r="B12" s="12" t="inlineStr">
-        <is>
-          <t>FR-CL-016</t>
-        </is>
-      </c>
-      <c r="C12" s="12" t="inlineStr">
-        <is>
-          <t>The meaning of the claims authorization code and any TL / TH override are open (CLQ01); the FRS tests only that the button is disabled while premium is unpaid.</t>
-        </is>
-      </c>
-      <c r="D12" s="12" t="inlineStr">
-        <is>
           <t>Answer CLQ01 before UAT and add the override case if one is agreed.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:D12"/>
+  <autoFilter ref="A4:D11"/>
   <mergeCells count="1">
     <mergeCell ref="A2:D2"/>
   </mergeCells>
-  <conditionalFormatting sqref="A5:D512">
+  <conditionalFormatting sqref="A5:D511">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>AND(MOD(ROW(),2)=0,$A5&lt;&gt;"")</formula>
     </cfRule>
@@ -3276,7 +3254,7 @@
       </c>
       <c r="E10" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F10" s="12" t="inlineStr">
@@ -3308,7 +3286,7 @@
       </c>
       <c r="E11" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F11" s="12" t="inlineStr">
@@ -3340,7 +3318,7 @@
       </c>
       <c r="E12" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F12" s="12" t="inlineStr">
@@ -3372,7 +3350,7 @@
       </c>
       <c r="E13" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F13" s="12" t="inlineStr">
@@ -3500,7 +3478,7 @@
       </c>
       <c r="E17" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F17" s="12" t="inlineStr">
@@ -3532,7 +3510,7 @@
       </c>
       <c r="E18" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F18" s="12" t="inlineStr">
@@ -3564,7 +3542,7 @@
       </c>
       <c r="E19" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F19" s="12" t="inlineStr">
@@ -3596,7 +3574,7 @@
       </c>
       <c r="E20" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F20" s="12" t="inlineStr">
@@ -3788,7 +3766,7 @@
       </c>
       <c r="E26" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F26" s="12" t="inlineStr">
@@ -3820,7 +3798,7 @@
       </c>
       <c r="E27" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F27" s="12" t="inlineStr">
@@ -3852,7 +3830,7 @@
       </c>
       <c r="E28" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F28" s="12" t="inlineStr">
@@ -3884,7 +3862,7 @@
       </c>
       <c r="E29" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F29" s="12" t="inlineStr">
@@ -3916,7 +3894,7 @@
       </c>
       <c r="E30" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F30" s="12" t="inlineStr">
@@ -3948,7 +3926,7 @@
       </c>
       <c r="E31" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F31" s="12" t="inlineStr">
@@ -3980,7 +3958,7 @@
       </c>
       <c r="E32" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F32" s="12" t="inlineStr">
@@ -4012,7 +3990,7 @@
       </c>
       <c r="E33" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F33" s="12" t="inlineStr">
@@ -4044,7 +4022,7 @@
       </c>
       <c r="E34" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F34" s="12" t="inlineStr">
@@ -4172,7 +4150,7 @@
       </c>
       <c r="E38" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F38" s="12" t="inlineStr">
@@ -4204,7 +4182,7 @@
       </c>
       <c r="E39" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F39" s="12" t="inlineStr">
@@ -4236,7 +4214,7 @@
       </c>
       <c r="E40" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F40" s="12" t="inlineStr">
@@ -4268,7 +4246,7 @@
       </c>
       <c r="E41" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F41" s="12" t="inlineStr">
@@ -4300,7 +4278,7 @@
       </c>
       <c r="E42" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F42" s="12" t="inlineStr">
@@ -4780,7 +4758,7 @@
       </c>
       <c r="E57" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F57" s="12" t="inlineStr">
@@ -4812,7 +4790,7 @@
       </c>
       <c r="E58" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F58" s="12" t="inlineStr">
@@ -4844,7 +4822,7 @@
       </c>
       <c r="E59" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F59" s="12" t="inlineStr">
@@ -4876,7 +4854,7 @@
       </c>
       <c r="E60" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F60" s="12" t="inlineStr">
@@ -4908,7 +4886,7 @@
       </c>
       <c r="E61" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F61" s="12" t="inlineStr">
@@ -4940,7 +4918,7 @@
       </c>
       <c r="E62" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F62" s="12" t="inlineStr">
@@ -4972,7 +4950,7 @@
       </c>
       <c r="E63" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F63" s="12" t="inlineStr">
@@ -5004,7 +4982,7 @@
       </c>
       <c r="E64" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F64" s="12" t="inlineStr">
@@ -5036,7 +5014,7 @@
       </c>
       <c r="E65" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F65" s="12" t="inlineStr">
@@ -5068,7 +5046,7 @@
       </c>
       <c r="E66" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F66" s="12" t="inlineStr">
@@ -5100,7 +5078,7 @@
       </c>
       <c r="E67" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F67" s="12" t="inlineStr">
@@ -5132,7 +5110,7 @@
       </c>
       <c r="E68" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F68" s="12" t="inlineStr">
@@ -5164,7 +5142,7 @@
       </c>
       <c r="E69" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F69" s="12" t="inlineStr">
@@ -5196,7 +5174,7 @@
       </c>
       <c r="E70" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F70" s="12" t="inlineStr">
@@ -5228,7 +5206,7 @@
       </c>
       <c r="E71" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F71" s="12" t="inlineStr">
@@ -5260,7 +5238,7 @@
       </c>
       <c r="E72" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F72" s="12" t="inlineStr">
@@ -5292,7 +5270,7 @@
       </c>
       <c r="E73" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F73" s="12" t="inlineStr">
@@ -5324,7 +5302,7 @@
       </c>
       <c r="E74" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F74" s="12" t="inlineStr">
@@ -5356,7 +5334,7 @@
       </c>
       <c r="E75" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F75" s="12" t="inlineStr">
@@ -5388,7 +5366,7 @@
       </c>
       <c r="E76" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F76" s="12" t="inlineStr">
@@ -5420,7 +5398,7 @@
       </c>
       <c r="E77" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F77" s="12" t="inlineStr">
@@ -5452,7 +5430,7 @@
       </c>
       <c r="E78" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F78" s="12" t="inlineStr">
@@ -5484,7 +5462,7 @@
       </c>
       <c r="E79" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F79" s="12" t="inlineStr">
@@ -5516,7 +5494,7 @@
       </c>
       <c r="E80" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F80" s="12" t="inlineStr">
@@ -5548,7 +5526,7 @@
       </c>
       <c r="E81" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F81" s="12" t="inlineStr">
@@ -5580,7 +5558,7 @@
       </c>
       <c r="E82" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F82" s="12" t="inlineStr">
@@ -5612,7 +5590,7 @@
       </c>
       <c r="E83" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F83" s="12" t="inlineStr">
@@ -5644,7 +5622,7 @@
       </c>
       <c r="E84" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F84" s="12" t="inlineStr">
@@ -5676,7 +5654,7 @@
       </c>
       <c r="E85" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F85" s="12" t="inlineStr">
@@ -5708,7 +5686,7 @@
       </c>
       <c r="E86" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F86" s="12" t="inlineStr">
@@ -5740,7 +5718,7 @@
       </c>
       <c r="E87" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F87" s="12" t="inlineStr">
@@ -5772,7 +5750,7 @@
       </c>
       <c r="E88" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F88" s="12" t="inlineStr">
@@ -5804,7 +5782,7 @@
       </c>
       <c r="E89" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F89" s="12" t="inlineStr">
@@ -5836,7 +5814,7 @@
       </c>
       <c r="E90" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F90" s="12" t="inlineStr">
@@ -5868,7 +5846,7 @@
       </c>
       <c r="E91" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F91" s="12" t="inlineStr">
@@ -5900,7 +5878,7 @@
       </c>
       <c r="E92" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F92" s="12" t="inlineStr">
@@ -5932,7 +5910,7 @@
       </c>
       <c r="E93" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F93" s="12" t="inlineStr">
@@ -5964,7 +5942,7 @@
       </c>
       <c r="E94" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F94" s="12" t="inlineStr">
@@ -5996,7 +5974,7 @@
       </c>
       <c r="E95" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F95" s="12" t="inlineStr">
@@ -6028,7 +6006,7 @@
       </c>
       <c r="E96" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F96" s="12" t="inlineStr">
@@ -6060,7 +6038,7 @@
       </c>
       <c r="E97" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F97" s="12" t="inlineStr">
@@ -6092,7 +6070,7 @@
       </c>
       <c r="E98" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F98" s="12" t="inlineStr">
@@ -6124,7 +6102,7 @@
       </c>
       <c r="E99" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F99" s="12" t="inlineStr">
@@ -6156,7 +6134,7 @@
       </c>
       <c r="E100" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F100" s="12" t="inlineStr">
@@ -6188,7 +6166,7 @@
       </c>
       <c r="E101" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F101" s="12" t="inlineStr">
@@ -6220,7 +6198,7 @@
       </c>
       <c r="E102" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F102" s="12" t="inlineStr">
@@ -6252,7 +6230,7 @@
       </c>
       <c r="E103" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F103" s="12" t="inlineStr">
@@ -6284,7 +6262,7 @@
       </c>
       <c r="E104" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F104" s="12" t="inlineStr">
@@ -6316,7 +6294,7 @@
       </c>
       <c r="E105" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F105" s="12" t="inlineStr">
@@ -6348,7 +6326,7 @@
       </c>
       <c r="E106" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F106" s="12" t="inlineStr">
@@ -6380,7 +6358,7 @@
       </c>
       <c r="E107" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F107" s="12" t="inlineStr">
@@ -6412,7 +6390,7 @@
       </c>
       <c r="E108" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F108" s="12" t="inlineStr">
@@ -6444,7 +6422,7 @@
       </c>
       <c r="E109" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F109" s="12" t="inlineStr">
@@ -6476,7 +6454,7 @@
       </c>
       <c r="E110" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F110" s="12" t="inlineStr">
@@ -6508,7 +6486,7 @@
       </c>
       <c r="E111" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F111" s="12" t="inlineStr">
@@ -6540,7 +6518,7 @@
       </c>
       <c r="E112" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F112" s="12" t="inlineStr">
@@ -6668,7 +6646,7 @@
       </c>
       <c r="E116" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F116" s="12" t="inlineStr">
@@ -6700,7 +6678,7 @@
       </c>
       <c r="E117" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F117" s="12" t="inlineStr">
@@ -6732,7 +6710,7 @@
       </c>
       <c r="E118" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F118" s="12" t="inlineStr">
@@ -6764,7 +6742,7 @@
       </c>
       <c r="E119" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F119" s="12" t="inlineStr">
@@ -6796,7 +6774,7 @@
       </c>
       <c r="E120" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F120" s="12" t="inlineStr">
@@ -6828,7 +6806,7 @@
       </c>
       <c r="E121" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F121" s="12" t="inlineStr">
@@ -6860,7 +6838,7 @@
       </c>
       <c r="E122" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F122" s="12" t="inlineStr">
@@ -6892,7 +6870,7 @@
       </c>
       <c r="E123" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F123" s="12" t="inlineStr">
@@ -6924,7 +6902,7 @@
       </c>
       <c r="E124" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F124" s="12" t="inlineStr">
@@ -6956,7 +6934,7 @@
       </c>
       <c r="E125" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F125" s="12" t="inlineStr">
@@ -6988,7 +6966,7 @@
       </c>
       <c r="E126" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F126" s="12" t="inlineStr">
@@ -7020,7 +6998,7 @@
       </c>
       <c r="E127" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F127" s="12" t="inlineStr">
@@ -7052,7 +7030,7 @@
       </c>
       <c r="E128" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F128" s="12" t="inlineStr">
@@ -7180,7 +7158,7 @@
       </c>
       <c r="E132" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F132" s="12" t="inlineStr">
@@ -7212,7 +7190,7 @@
       </c>
       <c r="E133" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F133" s="12" t="inlineStr">
@@ -7244,7 +7222,7 @@
       </c>
       <c r="E134" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F134" s="12" t="inlineStr">

</xml_diff>